<commit_message>
auto: session 2026-08-10 11:26
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/ke-hoach-noi-dung-cum-pr-2026-08-10.xlsx
+++ b/content/ke-hoach-noi-dung-cum-pr-2026-08-10.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Ke hoach bai viet" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Doi chieu cum" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Tu khoa chi tiet" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Ngoai pham vi" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Tu khoa chinh theo cum" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Ngoai pham vi" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,6 +103,10 @@
       <b val="1"/>
       <color rgb="00A85C10"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <b val="1"/>
@@ -186,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -241,13 +246,34 @@
     <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -338,6 +364,23 @@
     <tableColumn id="6" name="Cum"/>
     <tableColumn id="7" name="Trang thai"/>
     <tableColumn id="8" name="Trang / ghi chu"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TuKhoaChinhTheoCum" displayName="TuKhoaChinhTheoCum" ref="A1:H15" headerRowCount="1">
+  <autoFilter ref="A1:H15"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Cum tu khoa"/>
+    <tableColumn id="2" name="Tu khoa chinh (dai dien)"/>
+    <tableColumn id="3" name="Volume tu khoa chinh"/>
+    <tableColumn id="4" name="So tu khoa trong cum"/>
+    <tableColumn id="5" name="Tong volume cum"/>
+    <tableColumn id="6" name="Trang thai"/>
+    <tableColumn id="7" name="Trang / ghi chu"/>
+    <tableColumn id="8" name="Danh sach tu khoa con lai trong cum"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -632,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -836,7 +879,14 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Sheet 5 - Ngoai pham vi: 2 nhom tu khoa khong lien quan dich vu Digicom.</t>
+          <t>Sheet 5 - Tu khoa chinh theo cum: moi cum 1 dong - tu khoa chinh dai dien + toan bo tu khoa con lai trong cum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Sheet 6 - Ngoai pham vi: 2 nhom tu khoa khong lien quan dich vu Digicom.</t>
         </is>
       </c>
     </row>
@@ -23905,6 +23955,579 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Cum tu khoa</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Tu khoa chinh (dai dien)</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Volume tu khoa chinh</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>So tu khoa trong cum</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Tong volume cum</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Trang thai</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Trang / ghi chu</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Danh sach tu khoa con lai trong cum</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="46" customHeight="1">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Cách viết / công thức / cấu trúc</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>cấu trúc bài pr</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>290</v>
+      </c>
+      <c r="F2" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>/cach-viet-bai-pr-chuan-bao-chi/</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>cách viết bài pr; cách viết bài pr cho sản phẩm; cách viết bài pr sản phẩm; công thức viết bài pr; kỹ năng viết bài pr; bài pr theo công thức pas; các dạng bài pr; cách viết bài pr cho doanh nghiệp; cách viết bài pr trên facebook; viết bài pr theo công thức 3s; cách viết bài pr sự kiện; 12 cách viết tiêu đề cho bài pr; 3 công thức viết bài pr; bài pr bất động sản theo công thức; bài viết pr theo công thức 3s; bố cục bài pr; bố cục bài viết pr; bố cục một bài pr; các cách viết bài pr; các công thức viết bài pr; các dạng bài viết pr; các loại bài viết pr; cách viết 1 bài báo pr; cách viết 1 bài pr; cách viết 1 bài pr hiệu quả; cách viết 1 bài pr sản phẩm; cách viết bài báo pr; cách viết bài chia sẻ pr brand; cách viết bài pr cho công ty; cách viết bài pr cho mỹ phẩm; cách viết bài pr cho page; cách viết bài pr cho sản phẩm công nghệ; cách viết bài pr cho sự kiện; cách viết bài pr cho trung tâm ngoại ngữ; cách viết bài pr cho trường mầm non; cách viết bài pr chuyên đề; cách viết bài pr chương trình khuyến mãi; cách viết bài pr công ty; cách viết bài pr du lịch; cách viết bài pr dịch vụ; cách viết bài pr dự án bất động sản; cách viết bài pr giới thiệu sản phẩm; cách viết bài pr giới thiệu về workshop; cách viết bài pr hấp dẫn; cách viết bài pr khách sạn; cách viết bài pr lên báo; cách viết bài pr mỹ phẩm hiệu quả; cách viết bài pr ngược trong bds; cách viết bài pr nhân vật; cách viết bài pr pha t biê u; cách viết bài pr sách; cách viết bài pr theo công thức 3s; cách viết bài pr thuê; cách viết bài pr trên facebook group; cách viết bài pr trên fanpage hấp dẫn; cách viết bài pr về bệnh sỏi thận; cách viết bài pr về sản phẩm; cách viết bài pr đèn led; cách viết bài quản cáo pr trên facebook; cách viết bài quảng cáo pr trên facebook; cách viết bài truyền thông pr; cách viết một bài adaption trong pr; cấu trúc của một bài pr; học cách viết bài pr; kỹ năng viết bài pr bán hàng; kỹ năng viết bài pr fb; kỹ năng viết bài pr tăng doanh số bán hàng; phân loại bài pr; phân loại bài viết pr</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Đuôi dài chung (bài PR / viết bài PR...)</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>bài pr</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="D3" s="24" t="n">
+        <v>260</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="F3" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ gián tiếp (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>/bai-pr-la-gi/ + /cach-viet-bai-pr-chuan-bao-chi/ trả lời ở mức tổng quát</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>bài báo pr; bài viết pr; bài viết pr spa; viết bài pr; viết bài pr báo chí; 1 pr 2 4-9 bài đọc; 1 số bài viết pr son; 3 dang bài viết pr; 64 từ khóa trong viết bài pr; adverter bài pr; balo bài pr; bao gia bài pr báo saigon time; box thông tin bài pr; by-liner bài pr có qc chân trang; bài biết pr cho nội thất; bài báo pr chuyên; bài báo pr chuyên mục tài trợ tư vấn; bài báo pr thuộc công cụ quảng cáo nào; bài báo pr về sàn văn phòng; bài demographic trong pr; bài dịch về nhân viên pr; bài giảng pr truyền thông; bài học pr từ sunlight; bài pr 400 chữ; bài pr aroma resort trên dântrí bị xóa; bài pr bao nhiêu tiền; bài pr bia budweiser trên báo; bài pr budweiser trên báo; bài pr báo; bài pr báo chíu; bài pr báo lecourrier; bài pr báo saigon times online; bài pr cao sao vàng; bài pr cho công ty thiết kế nội thất; bài pr cho gà texas; bài pr cho page; bài pr cho texas; bài pr cho trang sức kim cương; bài pr có chèn tvc quảng cáo; bài pr của acnes; bài pr của kols viết như thế nào; bài pr demographic; bài pr gồm những phần nào; bài pr infographic; bài pr inforgraphic; bài pr kem chống nắng; bài pr kem đánh răng p s; bài pr khu đô thị; bài pr len; bài pr ly cafe; bài pr lửa trại; bài pr máy lọc khí sharp; bài pr nhà sách; bài pr nhân vật; bài pr nước hoa; bài pr nội bộ; bài pr saigon times; bài pr sách nguyễn nhật ánh; bài pr theo string; bài pr theo strings; bài pr tiếng anh là j; bài pr trên báo giúp tăng uy tín trên google; bài pr trên kênh14; bài pr trên thời báo kinh tế sài gòn; bài pr trưởng ban đối nội; bài pr tăng cơ bắp; bài pr tổng kết cuối nam; bài pr và bài quảng cáo; bài pr về bộ phận chăm sóc khách hàng; bài pr về ca sỹ; bài pr về công ty; bài pr về dasani; bài pr về digital marketing; bài pr về món nga; bài pr về nhân vật; bài pr về nutiboost; bài pr về nước dasani; bài pr về nước tẩy; bài pr về nước uống; bài pr về nội y; bài pr về phân bón; bài pr về sữa nutiboost; bài pr về trị mụn; bài pr về tập đoàn; bài pr xe tải; bài pr đơn vị tài trợ; bài pr đại lý; bài pr đại lý ô tô; bài viết cho báo chí và bài viết cho pr; bài viết chuẩn pr; bài viết pr branding cho bán lẻ; bài viết pr cho muối tôm tây ninh; bài viết pr cho shop; bài viết pr của now; bài viết pr của now.vn; bài viết pr do nhà báo viết; bài viết pr dạy bơi; bài viết pr fb; bài viết pr homestay; bài viết pr hài; bài viết pr layout; bài viết pr luxgarden; bài viết pr marketingai; bài viết pr nhân viên; bài viết pr nước hoa; bài viết pr quyên góp áo trắng cho em; bài viết pr sàn văn phòng; bài viết pr trà sữa; bài viết pr tôm hùm; bài viết pr vietnambiz; bài viết pr và quảng cáo khác nhau; bài viết pr về công ty; bài viết pr về durex; bài viết pr về nha trang; bài viết pr về đồ nội thất cao cấp; bài viết pr đồ ăn; bài viết quảng cáo pr; bài viết testimonal trong pr; bài đăng pr; bài đọc 2 1 pr 3 18-22; báo bài pr trên saigon tourist; báo bài pr trên saigontourist; bí quyết viết bài pr; cach viet một bài pr; caác bài phát biểu trong chiến dịch pr; caác bài pr cho dầu gội trị gàu; caác bài viết pr cho các dầu gội trị gàu; caácc bài pr cho dầu gội trị gàu; caách viết 1 bài pr; caách viết bài pr về công ty; caấu trúc một bài pr; chapeau bài pr; chiến lược đi bài pr; chèn clip vào bài pr; chủ đề viết bài pr; coông thức strings trong viết bài pr; các bài báo pr sacombank; các bài pr; các bài pr game; các bài pr nước hoa; các bài pr theo kiểu editorial; các bài pr về seo; các bài viết pr strings; các bài viết pr về bác sĩ hàn quốc; các bài viết pr về rong nho; các hình thức bài pr; các phần của bài viết pr; các thể loại bài viết pr; các viết bài pr; cách chuẩn bị bài phát biểu pr; cách lập dàn ý bài pr; cách thức viết 1 bài pr; cách thức viết bài pr; cách trình bày campaign trong báo cáo pr; cách xác định giai đoạn của môt bài pr; công cụ số liệu bài pr; cơ sở lý thuyết về bài pr của kols; cần người viết bài pr; cần tìm người viết bài pr; demo bài pr báo vne; diễn văn bài phát biểu trong pr; dàn ý một bài pr; dđặt bài viết pr; dđể viết tốt 1 bài pr; dđịnh nghĩa bài pr; dộ dài một bài pr; format bài pr gửi báo chí; format bài pr mớ; format bài pr mới; freelancer viết bài pr; gói bài pr cho seo; hoọc anh văn để viết bài pr; học viết bài pr; học viết bài pr marketing ở đâu; hợp đồng viết bài pr; khung viết một bài pr; khóa học viết bài pr; kinh nghiệm viết bài pr; kế hoạch tin bài pr; kế hoạch viết cho bài pr; kỹ thuật viết bài pr; kỹ thuật viết bài pr pdf; kỹ thuật viết bài pr quảng cáo pdf; làm sao để viết bài pr; lượt view trung bình cho bài pr hieeu; mua sách kỹ thuật viết bài pr; mô hình kim tự tháp ngược trong viết bài pr; nestle bài pr; neên đi bài pr như thế nào; nghiên cứu về bài pr; nghề viết bài pr; nghệ thuật viết bài pr; nguyên tắc viết bài pr; nguyên tắc viết bài pr trên báo chí; nhung bài viết pr bán nhà đất; nhân viên viết bài pr; nhận viết bài pr; những bài pr nổi tiếng; những bài pr nổi tiếng fb; những bài pr đăng cuối năm; những bài viết pr cho ngày hội sách; những bài viết pr cho trung tâm tiếng anh; phân biệt 1 bài báo và 1 bài pr; phân biệt bài viết pr; phân cấp bài pr; phân tích một bài pr trên báo; phần mở đầu của một bài pr; pr là hãng bày nào; quy cách đi bài pr trên báo; sabo bài pr; sách kỹ thuật viết bài pr quảng cáo; sườn bài pr; thế nào là bài báo pr; tiêu chí của một bài pr; tiêu đề bài pr; toplist.vn là trang web viết các bài pr lừa đảo; trình bày các công cụ của pr; trình bày khái niệm pr; tìm người viết bài pr; tìm người viết bài pr fb; tìm từ khóa trên bài viết pr onliine; tìm từ khóa trên bài viết pr online; tìm việc làm viết bài pr; từ khóa seo cho bài pr; unica kĩ thuật viết bài pr quảng cáo; vieế bài pr theo cong thức strings; vieết bài pr sao cho thu hút; vieết bài pr tại nhà; viết bài pr bao nhiêu tiền 1 bài; viết bài pr chia sẻ lên các diễn đàn; viết bài pr cho cảng biển; viết bài pr cho phụ gia ngành giấy; viết bài pr cho studio cưới; viết bài pr công ty; viết bài pr công ty honda; viết bài pr công ty với 200 từ; viết bài pr first sight; viết bài pr hiệu quả; viết bài pr la gì; viết bài pr món ăn cho người mới bắt đầu; viết bài pr toeic; viết bài pr và seo; viết bài pr về món nga; viết bài pr về địa điểm tổ chức; viết bài pr zalo; viết bài pr đăng báo; viết bài quảng pr cho phân bón; viết kết bài pr; văn phong bài pr; vị trí pr bài viết trên báo điện tử; xem báo giaá bài pr các báo ở đâu; xem số liệu bài pr; xu hướng viết bài pr; xác định công chúng của bài viết pr; xây dựng thông điệp của bài viết pr; yêu cầu của một bài pr; yý tưởng viết bài pr; đặt tít bài pr sao cho hấp dẫn; đọc &amp; phân tích các bài pr sau</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Mẫu / ví dụ bài PR</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>bài pr mẫu</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" s="24" t="n">
+        <v>67</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>/bai-pr-mau/</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>bài pr hay; các bài pr mẫu; mẫu bài viết pr sự kiện; những bài pr hay; những bài viết pr sản phẩm hay; những mẫu bài pr hay; bài viết pr mẫu; các bài pr hay; mẫu bài pr sản phẩm; bài mẫu pr; bài mẫu pr sự kiện; bài mẫu pr về món nga; bài pr mẫu của tổ chức giáo dục; bài pr mẫu theo công thức pas; bài pr mẫu về công ty; bài pr mẫu về nhân vật; bài pr nhà hangfd hay; bài pr nhân vật hay; bài pr sản phẩm hay; bài pr sản phẩm mẫu; bài viết pr hay; bài viết pr mẫu xe hơi; bài viết pr sản phẩm mẫu; bài viết pr về sản phẩm hay; caách giật tít hay cho bài pr; các bài phỏng pr vấn mẫu; các bài pr hay về dược phẩm; các bài pr pas mẫu; các bài pr sự kiện mẫu; các bài viết pr sản phẩm hay; các facebooer viết pr bài viết hay; các facebooker viết pr bài viết hay; các facebooker viết pr bài viết hay nổi tiếng; các nhân vật viết pr bài viết hay; cách giật tít hay cho bài pr; cách nhận biết baì pr hay bài marketing; cách tạo một bài pr hay; cách viết bài pr hay; cách viết bài pr sản phẩm hay; mẫu 1 bài pr; mẫu bài pr cho sự kiện; mẫu bài pr hay; mẫu bài pr theo aida; mẫu bài pr theo công thức aida; mẫu bài pr xe tải; mẫu bài viết pr sản phẩm; một bài pr mẫu cho ra mắt sản phẩm mới; một bài pr ấn tượng; một số bài pr hay; một số bài pr mẫu; một số bài pr mẫu sự kiện; nhung bài viết pr bán nhà đất hay; những bài pr game hay; những bài pr hay nhất; những bài pr hầm rượu vang hay; những bài pr pas mẫu; những bài viết pr hay; những bài viết pr hay nhất; những bài viết pr về shop hay; tham khảo các mẫu bài pr đỉnh cao; tập hợp các bài viết hay về pr; ví dụ bài pr; ví dụ các bài pr về món nga; ví dụ các công thức viết bài pr; ví dụ các công thức viết bài pr facebook; đặt tít hay cho bài pr sản phẩm sơn</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>Báo giá theo đầu báo cụ thể</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>báo giá bài pr vnexpress</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>152</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="F5" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm Booking báo)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>15 trang /book-bao-*/ + /booking-bao-pr/</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>báo giá đăng bài pr trên kenh14; báo giá bài pr 24h; báo giá bài pr cafef; báo giá bài pr kenh14; báo giá bài pr trên vnexpress; báo giá bài pr vietnamnet; báo giá đăng bài pr trên kênh 14; báo giá đăng bài pr trên vnexpress; agency book bài pr trên báo cnn; agency book bài pr trên times new; bao gia bài pr giaoduc.net.vn; bao giaá viết bài pr cafef; bao giá bài pr báo xa luan điện tử; bao giá bài pr theleader; bao giá bài pr thế giới tiếp thị online; bao giá bài pr xa luan online; bao giá bài pr xaluan online; baáo giá bài pr an ninh thủ đô online; baáo giá bài pr baodautu.vn; baáo giá bài pr báo thanh niên online; baáo giá bài pr báo đầu tư; baáo giá bài pr báo đầu tư 2019; baáo giá bài pr eva; baáo giá bài pr người lao động; baáo giá bài pr thiếu niên tiền phong online; baáo giá bài pr tiếp thị gia đình báo giấy; baáo giá bài pr trên báo baodautu.vn; baáo giá bài pr vietnam economic times online; baáo giá bài pr vietnamnet; baáo giá bài pr vir online; baáo giá bài pr vnexpress; baáo giá bài pr zing news; baáo giá lên bài pr 24h.com.vn; baáo giá lên bài pr afamily.vn; baáo giá lên bài pr baodautu.vn; baáo giá lên bài pr batdongsan.com.vn; baáo giá lên bài pr cafebiz; baáo giá lên bài pr cafef; baáo giá lên bài pr dân trí; baáo giá lên bài pr eva.vn; baáo giá lên bài pr giadinh.net; baáo giá lên bài pr ictnew; baáo giá lên bài pr otofun; baáo giá lên bài pr soha; baáo giá lên bài pr thanh niên; baáo giá lên bài pr vietnamnet; baáo giá lên bài pr vnexpress; baáo giá lên bài pr zing; baáo giá đăng bài pr trên soha; book bài pr trên báo nước ngoài cnn; book bài pr trên tạp chí bác sĩ gia đình; booking bài pr báo batdongsan.com.vn; booking bài pr trên tiếp thị và gia đình; bài pr aroma resort trên dân trí bị xóa; bài pr báo msn online; bài pr báo pháp luật online; bài pr báo sggp hoa van online; bài pr báo sggp online; bài pr báo vtc news online; bài pr cafef; bài pr dân trí; bài pr kenh14; bài pr ngoisao; bài pr ngoisao.net; bài pr thanh niên; bài pr trên vnexpress; bài pr zing; báo giá book bài pr trên vnexpress; báo giá bài pr 24h.com.vn; báo giá bài pr afamily; báo giá bài pr báo công an giấy; báo giá bài pr báo công an nhân dân online; báo giá bài pr báo giấy sggp hoa văn; báo giá bài pr báo giấy tiếp thị gia đình; báo giá bài pr báo giấy tuổi trẻ; báo giá bài pr báo lao động online; báo giá bài pr báo pháp luật việt nam online; báo giá bài pr báo theleader; báo giá bài pr báo tiếp thị gia đình online; báo giá bài pr báo vnexpress; báo giá bài pr báo vtc điện tử; báo giá bài pr báo xaluan; báo giá bài pr báo đầu tư 2019; báo giá bài pr doanh nhân sài gòn; báo giá bài pr eva.vn; báo giá bài pr kenh14 2017; báo giá bài pr lao động online; báo giá bài pr ngoisao.net; báo giá bài pr người lao động; báo giá bài pr người lao động 2019; báo giá bài pr người lao động online; báo giá bài pr sài gòn giải phóng online; báo giá bài pr theleader; báo giá bài pr tiền phong online; báo giá bài pr trên 24h; báo giá bài pr trên afamily; báo giá bài pr trên baodautu.vn; báo giá bài pr trên báo baodautu.vn; báo giá bài pr trên dân trí; báo giá bài pr trên eva; báo giá bài pr trên eva.vn; báo giá bài pr trên lao động online; báo giá bài pr trên ngoisao net; báo giá bài pr trên vietnamnet; báo giá bài pr trên vnexpress 2017; báo giá bài pr trên vnexpress 2018; báo giá bài pr trên webtretho; báo giá bài pr trên zing; báo giá bài pr tạp chí elle; báo giá bài pr vietnam investment review online; báo giá bài pr vnexpress 2019; báo giá bài pr vnreview; báo giá bài pr vov; báo giá đăng bài pr batdongsan.com.vn; báo giá đăng bài pr trên 24h; báo giá đăng bài pr trên 24h.com.vn; báo giá đăng bài pr trên cafef; báo giá đăng bài pr trên soha; báo giá đăng bài pr trên zing; bảng giá đăng bài pr trên báo 24h; bảng giá đăng bài pr trên báo tuổi trẻ; cafef bài pr; cafef bài pr giá; chi phí bài pr của kenh14; chi phí thuê viết bài pr trên tạp chí elle; chi phí viết bài pr trên new zing; chi phí viết bài pr trên vnexpress; chi phí đăng bài pr trên cafebiz; chi phí đăng bài pr trên ictnews; cách thuê dân trí pr bài viết; demo các vị trí bài pr trên vnexpress; format bài pr gửi báo chí times new roman; giá book bài pr kenh14; giá bài pr trên dân trí; giá bài pr trên sggp hoa van dien tử; giá bài pr trên thời sự vtv1; giá bài pr trên vnexpress; giá bài pr tạp chí tài chính; giá bài quảng cáo pr baomoi.com; giá bài quảng cáo pr new.zing.vn; giá bài viết pr trên zing; giá đăng bài pr vnexpress 2017; liên hệ bài pr trên vnexpress; lên bài pr baomoi; viết bài pr trên báo cafef; đăng bài pr trên báo dân trí; đăng bài pr trên cafef; đăng bài pr trên eva.vn; đăng bài pr trên giadinh.net; đăng bài pr trên vietnamnet; đăng bài pr trên vnexpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Dịch vụ viết bài PR (chưa có trang)</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>dịch vụ viết bài pr</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>160</v>
+      </c>
+      <c r="F6" s="26" t="inlineStr">
+        <is>
+          <t>Gap - BÀI MỚI (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Đề xuất bài mới, CTA về /booking-bao-pr/</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>báo giá viết bài pr; chi phí viết bài pr; thuê viết bài pr; giá viết bài pr; báo giá bài viết pr trên website cho phu nư; báo giá dịch vụ viết bài pr; báo giá viết bài pr cho sản phẩm; báo giá viết bài pr trên http genk.vn; bảng báo giá viết bài pr trên baogiaothong.vn; bảng giá viết bài pr; cách đánh giá bài viết pr hiệu quả; dịch vụ viết bài pr chuyên nghiệp; gía dịch vụ viết bài pr</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Giá / đăng / booking chung (không kèm tên báo)</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>đăng bài pr</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <v>126</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>130</v>
+      </c>
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm Booking báo)</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>/booking-bao-pr/ (hub giá)</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>book bài pr; báo giá bài pr; giá bài pr; giá đăng bài pr; booking bài pr; đăng bài pr trên báo; agency book bài pr; agency book bài pr trên các báo nước ngoài; agency book bài pr được các báo online nước ngoài; agency đăng bài pr; bao giá bài pr dmtin; baáo giá bài pr; baáo giá bài pr báo vsao; baáo giá bài pr báo vsao điện tử; baáo giá bài pr báo xã luận điện tử; baáo giá bài pr dantri; baáo giá gói đăng bài pr trên ngôi sao.net; baáo giá lên bài pr phunuonline; baáo giá lên bài pr thethaovanhoa; baáo giá lên bài pr tuoitre; baáo giá lên bài pr vietnamexpress; baáo giá lên bài pr vneconomy; biểu giá bài pr báo công thương online; biểu giá bài pr báo công thương điện tử; book bài pr admicro; book bài pr trên báo nước ngoài time; booking bài pr báo online; booking viết bài pr; báo giá booking bài pr admicro; báo giá bài pr báo công thương online; báo giá bài pr báo hoa học trò điện tử; báo giá bài pr báo ione; báo giá bài pr báo mtv; báo giá bài pr báo mtv we điện tử; báo giá bài pr báo mtvwe điện tử; báo giá bài pr báo thitkho; báo giá bài pr báo thê thao văn hóa online; báo giá bài pr báo vsao.com; báo giá bài pr báo xone điện tử; báo giá bài pr bạch mỹ liên; báo giá bài pr chính phủ online; báo giá bài pr dan ong magazine; báo giá bài pr dantri.com.vn; báo giá bài pr dantri.com.vn 2017; báo giá bài pr ict news; báo giá bài pr ione 2017; báo giá bài pr kenh 14; báo giá bài pr marrybaby; báo giá bài pr online; báo giá bài pr thanhnien; báo giá bài pr the leader; báo giá bài pr thế giới văn hóa online; báo giá bài pr trên báo giấy lao độn; báo giá bài pr trên báo mới; báo giá bài pr trên doanh nhan cuoi tuan online; báo giá bài pr trên doanh nhan plus; báo giá bài pr trên foody; báo giá bài pr trên kienthuc; báo giá bài pr trên kienthucdoisong; báo giá bài pr trên marrybaby; báo giá bài pr trên thanhnien.vn; báo giá bài pr trên thế giới văn hóa; báo giá bài pr trên thế giới văn hóa online; báo giá bài pr trên trang thegioivanhoa.net; báo giá bài pr trên trang thế giới văn hóa.net; báo giá bài pr trên trang voh; báo giá bài pr tư vấn tiêu dùng; báo giá bài pr tư vấn tiêu dùng online; báo giá bài pr v economic times online; báo giá bài pr vneconomy online; báo giá bài pr vo; báo giá bài pr voh; báo giá bài pr đàn ông magazine; báo giá đăng bài pr trên baoquocte.vn; báo giá đăng bài pr trên báo quốc tế; bảng giá book bài pr trên ivivu; bảng giá bài pr có chèn tvc quảng cáo; bảng giá đăng bài pr trên báo điện tử; bảng giá đăng bài pr vneconomy; cah đăng bài pr trên các trang báo điện tử; chi phi đăng bài pr trên các báo; chi phí book bài pr; chuỗi bài pr giá rẻ; các bài pr mảng giáo dục; cách book bài pr trên báo chí; cách viêt bài pr facebook cho sản phẩm; cách đăng bài pr trên báo chí; công ty booking bài pr; giá 1 bài pr thông thường; giá 1 bài pr trên elle.vn; giá 1 bài pr trên kenh 14; giá bài pr báo công thương online; giá bài pr báo lecourrier; giá bài pr báo lecourrier online; giá bài pr forbes; giá bài pr trên báo bưu điện; giá bài pr trên báo đẹp plus điện tử; giá bài pr trên depplus online; giá bài pr trên docbao online; giá bài pr trên thời báo kinh tế; giá bài pr trên trang infonet online; giá bài quảng cáo pr basomoi.com; giá bài quảng cáo pr trên autobikes.vn; giá bài quảng cáo pr trên tinxe.vn; giá bài viêt pr trên diadiemanuong; giá chạy bài pr trên vneconomy là bao nhiêu; giá của một bài pr trung bình hiện nay; giá dang bài pr báo mới; giá đăng bài pr trên báo điện tử; giá đăng bài pr trên các báo; gói mua bài pr giá rẻ; hệ thống book bài pr trên các báo; hỗ trợ đăng bài pr trên nhịp sống sendo; kênh đăng bài pr; neên đăng bài pr lên báo nào; những bài pr dịch vụ educate consumers; viết bài pr facebook; viết bài pr sản phẩm trên facebook; viết bài pr thuê; xem báo giá bài pr các báo ở đâu; đăng bài pr báo điện tử; đăng bài pr trên báo điện tử; đăng bài pr trên các báo lớn; đăng bài pr trên phụ nữ today; đăng bài pr ở đâu</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>PR theo sản phẩm</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>bài pr sản phẩm mới</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>110</v>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Mục con trong /cach-viet-bai-pr-chuan-bao-chi/ + /bai-pr-mau/</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>bài viết pr sản phẩm; bài viết pr về sản phẩm; viết bài pr cho sản phẩm; viết bài pr sản phẩm; bài biết pr cho sản phẩm nước giải khát; bài pr cho sản phẩm; bài pr cho sản phẩm dành cho pg; bài pr cho sản phẩm mới ra mắt; bài viết pr cho sản phẩm nước giải khát; bài viết pr sản phẩm của học vien; cau trúc viêt bài pr sản phẩm; các bài viết pr sản phẩm; các bài viết pr sản phẩm handmade; cách làm 1 bài pr cho 1 sản phẩm; neên đăn bài pr sản phẩm trên báo nào; sản phẩm mới của samsung bài pr; tieu đề bài pr giới thiệu sản phẩm; viết bài pr sản phẩm kiếm tiền; viết bài pr sản phẩm mới; viết bài pr sản phẩm thu hút khách hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>PR doanh nghiệp / thương hiệu</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>bài pr thương hiệu</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>/bai-pr-mau/</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>bài pr doanh nghiệp; bài pr cho doanh nghiệp; viết bài pr cho doanh nghiệp; bài pr từ thương hiệu; bài pr về doanh nghiệp; bài viết pr doanh nghiệp may mặc; bài viết pr tăng độ nhận diện thương hiệu; có được bán bài pr doanh nghiệp không; hướng dẫn viết bài pr cho doanh nghiệp; nguyeên tắc iets một bài pr thương hiệu; viết bài pr cho thương hiệu cho doanh nghiệp; viết bài pr cho thương hiệu công ty con; viết bài pr cho thương hiệu giày nike; viết bài pr doanh nghiệp</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>Định nghĩa "bài PR là gì"</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>viết bài pr là gì</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>/bai-pr-la-gi/</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>bài pr là gì; bài pr có chân dung quảng cáo là gì; bài pr có chân dung quảng cáo là gì marketing; bài viết pr tiếng anh là gì; diễn văn bài phát biểu là gì trong pr; lead bài pr là gì; sabo là gì trong viết bài pr; viết bài pr editorial là gì; viết bài pr nghĩa là gì; đăng bài pr là gì</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Mẫu/ví dụ theo ngành (chưa có)</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>bài viết pr về du lịch</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Thêm chip-grid ngành vào /bai-pr-mau/</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>bài pr về nhà hàng; bài viết pr khách sạn; bài pr cho bất động sản; bài pr cực hay về nhà hàng; bài pr mỹ phẩm; bài pr về nhà hàng nga tại việt nam; bài viết pr du lịch cần những gì; bài viết pr khu du lịch sinh thái; bài viết pr khách sạn mẫu; bài viết pr một khu du lịch; bài viết pr nhà hàng; bài viết pr nhà hàng trên báo mạng; các bài pr cho một chương trình bất động sản; mẫu bài pr bất động sản theo công thức; mẫu bài viết pr về khách sạn; tiêu chí bài pr bất động sản hay; top bài pr bất động sản đặc sắc; vieết bài pr cho khách sạn</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>Viết bài PR chuẩn SEO</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>viết bài pr chuẩn seo</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Thêm mục vào /cach-viet-bai-pr-chuan-bao-chi/, link /mua-textlink/ + /dich-vu-backlink/</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>cách viết bài pr chuẩn seo; dịch viết bài pr chuẩn seo; dịch vụ viết bài pr chuẩn seo; kỹ năng viết bài pr chuẩn seo; kỹ năng viết bài pr chuẩn seo ebook; seongon checklist bài pr chuẩn seo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>PR bản thân / xin việc (Jiko PR)</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>bài mẫu pr bản thân bằng tiếng nhật</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>bài pr bản thân; bài pr bản thân bằng tiếng nhật; bài viết pr bản thân; bài viết pr về bản thân; các bài viết pr cho game học tiếng nhật; nhờ các facebook cá nhân viết bài pr; yêu cầu về bài pr cá nhân</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>CTV / tuyển người viết</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>ctv viết bài pr</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>Ngoài phạm vi</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>cộng tác viên viết bài pr; agency tuyển ctv viết bài pr; agency tuyển team viết bài pr; agency tuyển viết bài pr; mục đích đăng bài tuyển dụng để pr; tuyển ctv viết bài pr; tuyển ctv viết bài pr báo chí; tuyển cộng tác viên viết bài pr; tuyển người viết bài pr; tuyển nhân viên pr viết bài website; tuyển viết bài pr agency; tuyển viết bài pr đăng báo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>PR theo sự kiện</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>viết bài pr cho sự kiện</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Mục con trong /bai-pr-mau/</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>bài pr sau sự kiện; bài pr sự kiện; bài pr sự kiện về quốc tế thiếu nhi; bài viết pr sự kiện; bài viết pr sự kiện ô tô; caác bài viết pr sự kiện; caách viết bài pr sự kiện; các bài viết pr cho sự kiện; những bài viết pr cho sự kiện ngày hội sách</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -23914,63 +24537,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>NGOAI PHAM VI - KHONG VIET, KHONG GOP</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>PR bản thân / xin việc (Jiko PR)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>8 tu khoa - 20 luot/thang</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>Vi du: bài mẫu pr bản thân bằng tiếng nhật, bài pr bản thân, bài pr bản thân bằng tiếng nhật, bài viết pr bản thân, bài viết pr về bản thân, các bài viết pr cho game học tiếng nhật, nhờ các facebook cá nhân viết bài pr, yêu cầu về bài pr cá nhân</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>CTV / tuyển người viết</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>13 tu khoa - 20 luot/thang</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t>Vi du: ctv viết bài pr, cộng tác viên viết bài pr, agency tuyển ctv viết bài pr, agency tuyển team viết bài pr, agency tuyển viết bài pr, mục đích đăng bài tuyển dụng để pr, tuyển ctv viết bài pr, tuyển ctv viết bài pr báo chí, tuyển cộng tác viên viết bài pr, tuyển người viết bài pr</t>
         </is>

</xml_diff>

<commit_message>
auto: session 2026-08-10 11:36
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/ke-hoach-noi-dung-cum-pr-2026-08-10.xlsx
+++ b/content/ke-hoach-noi-dung-cum-pr-2026-08-10.xlsx
@@ -874,7 +874,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>16</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Viet 1 bai rieng ve quy trinh viet (Digicom viet hay khach tu viet), viet mien phi khi dat tu 3 dau bao (dung uu dai hien co), chi phi neu viet rieng. CTA chinh dan ve /booking-bao-pr/. Duoc link vao tu /bai-pr-la-gi/ va /cach-viet-bai-pr-chuan-bao-chi/.</t>
+          <t>Viet 1 bai rieng ve quy trinh viet (Digicom viet hay khach tu viet), viet mien phi khi dat tu 3 dau bao (dung uu dai hien co), chi phi neu viet rieng. Neu them 1 doan cho doi tuong 'PR ca nhan/doanh nhan' (Hieu xac nhan day la nhu cau thuc: nguoi muon booking bao de PR cho chinh minh, khong phai viet CV xin viec - tu khoa 'bai pr ban than/ca nhan'). CTA chinh dan ve /booking-bao-pr/. Duoc link vao tu /bai-pr-la-gi/ va /cach-viet-bai-pr-chuan-bao-chi/.</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1500,11 +1500,11 @@
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
+          <t>PR bản thân - xin việc/du học Nhật (Jiko PR)</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C13" s="11" t="n">
         <v>20</v>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
@@ -1569,21 +1569,44 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
           <t>Nhiễu (loại)</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B17" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Loại</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2281,7 +2304,7 @@
       <c r="E20" s="17" t="inlineStr"/>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
+          <t>PR bản thân - xin việc/du học Nhật (Jiko PR)</t>
         </is>
       </c>
       <c r="G20" s="20" t="inlineStr">
@@ -2291,7 +2314,7 @@
       </c>
       <c r="H20" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
@@ -6761,17 +6784,17 @@
       <c r="E180" s="17" t="inlineStr"/>
       <c r="F180" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
-        </is>
-      </c>
-      <c r="G180" s="20" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="G180" s="21" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
         </is>
       </c>
       <c r="H180" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
@@ -6789,7 +6812,7 @@
       <c r="E181" s="17" t="inlineStr"/>
       <c r="F181" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
+          <t>PR bản thân - xin việc/du học Nhật (Jiko PR)</t>
         </is>
       </c>
       <c r="G181" s="20" t="inlineStr">
@@ -6799,7 +6822,7 @@
       </c>
       <c r="H181" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
@@ -9337,17 +9360,17 @@
       <c r="E272" s="17" t="inlineStr"/>
       <c r="F272" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
-        </is>
-      </c>
-      <c r="G272" s="20" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="G272" s="21" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
         </is>
       </c>
       <c r="H272" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
@@ -10401,17 +10424,17 @@
       <c r="E310" s="17" t="inlineStr"/>
       <c r="F310" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
-        </is>
-      </c>
-      <c r="G310" s="20" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="G310" s="21" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
         </is>
       </c>
       <c r="H310" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
@@ -15133,7 +15156,7 @@
       <c r="E479" s="17" t="inlineStr"/>
       <c r="F479" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
+          <t>PR bản thân - xin việc/du học Nhật (Jiko PR)</t>
         </is>
       </c>
       <c r="G479" s="20" t="inlineStr">
@@ -15143,7 +15166,7 @@
       </c>
       <c r="H479" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
@@ -20593,17 +20616,17 @@
       <c r="E674" s="17" t="inlineStr"/>
       <c r="F674" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
-        </is>
-      </c>
-      <c r="G674" s="20" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="G674" s="21" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
         </is>
       </c>
       <c r="H674" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
@@ -23533,17 +23556,17 @@
       <c r="E779" s="17" t="inlineStr"/>
       <c r="F779" s="15" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
-        </is>
-      </c>
-      <c r="G779" s="20" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="G779" s="21" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
         </is>
       </c>
       <c r="H779" s="17" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
@@ -43911,7 +43934,7 @@
     <row r="764">
       <c r="A764" s="22" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
+          <t>PR bản thân - xin việc/du học Nhật (Jiko PR)</t>
         </is>
       </c>
       <c r="B764" s="23" t="inlineStr">
@@ -43934,7 +43957,7 @@
       </c>
       <c r="F764" s="26" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
@@ -43947,7 +43970,7 @@
       </c>
       <c r="C765" s="32" t="inlineStr">
         <is>
-          <t>bài pr bản thân</t>
+          <t>bài pr bản thân bằng tiếng nhật</t>
         </is>
       </c>
       <c r="D765" s="33" t="n">
@@ -43960,12 +43983,12 @@
       </c>
       <c r="F765" s="34" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
     <row r="766">
-      <c r="A766" s="27" t="n"/>
+      <c r="A766" s="31" t="n"/>
       <c r="B766" s="32" t="inlineStr">
         <is>
           <t>—</t>
@@ -43973,7 +43996,7 @@
       </c>
       <c r="C766" s="32" t="inlineStr">
         <is>
-          <t>bài pr bản thân bằng tiếng nhật</t>
+          <t>các bài viết pr cho game học tiếng nhật</t>
         </is>
       </c>
       <c r="D766" s="33" t="n">
@@ -43986,75 +44009,79 @@
       </c>
       <c r="F766" s="34" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
     <row r="767">
-      <c r="A767" s="27" t="n"/>
-      <c r="B767" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C767" s="32" t="inlineStr">
-        <is>
-          <t>bài viết pr bản thân</t>
-        </is>
-      </c>
-      <c r="D767" s="33" t="n">
-        <v>0</v>
+      <c r="A767" s="22" t="inlineStr">
+        <is>
+          <t>CTV / tuyển người viết</t>
+        </is>
+      </c>
+      <c r="B767" s="23" t="inlineStr">
+        <is>
+          <t>Từ khoá chính</t>
+        </is>
+      </c>
+      <c r="C767" s="23" t="inlineStr">
+        <is>
+          <t>ctv viết bài pr</t>
+        </is>
+      </c>
+      <c r="D767" s="24" t="n">
+        <v>10</v>
       </c>
       <c r="E767" s="37" t="inlineStr">
         <is>
           <t>Ngoài phạm vi</t>
         </is>
       </c>
-      <c r="F767" s="34" t="inlineStr">
-        <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+      <c r="F767" s="26" t="inlineStr">
+        <is>
+          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
       </c>
     </row>
     <row r="768">
       <c r="A768" s="27" t="n"/>
-      <c r="B768" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C768" s="32" t="inlineStr">
-        <is>
-          <t>bài viết pr về bản thân</t>
-        </is>
-      </c>
-      <c r="D768" s="33" t="n">
-        <v>0</v>
+      <c r="B768" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C768" s="28" t="inlineStr">
+        <is>
+          <t>cộng tác viên viết bài pr</t>
+        </is>
+      </c>
+      <c r="D768" s="29" t="n">
+        <v>10</v>
       </c>
       <c r="E768" s="37" t="inlineStr">
         <is>
           <t>Ngoài phạm vi</t>
         </is>
       </c>
-      <c r="F768" s="34" t="inlineStr">
-        <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+      <c r="F768" s="30" t="inlineStr">
+        <is>
+          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
       </c>
     </row>
     <row r="769">
       <c r="A769" s="27" t="n"/>
-      <c r="B769" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C769" s="32" t="inlineStr">
-        <is>
-          <t>các bài viết pr cho game học tiếng nhật</t>
-        </is>
-      </c>
-      <c r="D769" s="33" t="n">
+      <c r="B769" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C769" s="28" t="inlineStr">
+        <is>
+          <t>agency tuyển ctv viết bài pr</t>
+        </is>
+      </c>
+      <c r="D769" s="29" t="n">
         <v>0</v>
       </c>
       <c r="E769" s="37" t="inlineStr">
@@ -44062,25 +44089,25 @@
           <t>Ngoài phạm vi</t>
         </is>
       </c>
-      <c r="F769" s="34" t="inlineStr">
-        <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+      <c r="F769" s="30" t="inlineStr">
+        <is>
+          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
       </c>
     </row>
     <row r="770">
       <c r="A770" s="27" t="n"/>
-      <c r="B770" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C770" s="32" t="inlineStr">
-        <is>
-          <t>nhờ các facebook cá nhân viết bài pr</t>
-        </is>
-      </c>
-      <c r="D770" s="33" t="n">
+      <c r="B770" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C770" s="28" t="inlineStr">
+        <is>
+          <t>agency tuyển team viết bài pr</t>
+        </is>
+      </c>
+      <c r="D770" s="29" t="n">
         <v>0</v>
       </c>
       <c r="E770" s="37" t="inlineStr">
@@ -44088,25 +44115,25 @@
           <t>Ngoài phạm vi</t>
         </is>
       </c>
-      <c r="F770" s="34" t="inlineStr">
-        <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+      <c r="F770" s="30" t="inlineStr">
+        <is>
+          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
       </c>
     </row>
     <row r="771">
-      <c r="A771" s="31" t="n"/>
-      <c r="B771" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C771" s="32" t="inlineStr">
-        <is>
-          <t>yêu cầu về bài pr cá nhân</t>
-        </is>
-      </c>
-      <c r="D771" s="33" t="n">
+      <c r="A771" s="27" t="n"/>
+      <c r="B771" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C771" s="28" t="inlineStr">
+        <is>
+          <t>agency tuyển viết bài pr</t>
+        </is>
+      </c>
+      <c r="D771" s="29" t="n">
         <v>0</v>
       </c>
       <c r="E771" s="37" t="inlineStr">
@@ -44114,37 +44141,33 @@
           <t>Ngoài phạm vi</t>
         </is>
       </c>
-      <c r="F771" s="34" t="inlineStr">
-        <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+      <c r="F771" s="30" t="inlineStr">
+        <is>
+          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
       </c>
     </row>
     <row r="772">
-      <c r="A772" s="22" t="inlineStr">
-        <is>
-          <t>CTV / tuyển người viết</t>
-        </is>
-      </c>
-      <c r="B772" s="23" t="inlineStr">
-        <is>
-          <t>Từ khoá chính</t>
-        </is>
-      </c>
-      <c r="C772" s="23" t="inlineStr">
-        <is>
-          <t>ctv viết bài pr</t>
-        </is>
-      </c>
-      <c r="D772" s="24" t="n">
-        <v>10</v>
+      <c r="A772" s="27" t="n"/>
+      <c r="B772" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C772" s="28" t="inlineStr">
+        <is>
+          <t>mục đích đăng bài tuyển dụng để pr</t>
+        </is>
+      </c>
+      <c r="D772" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="E772" s="37" t="inlineStr">
         <is>
           <t>Ngoài phạm vi</t>
         </is>
       </c>
-      <c r="F772" s="26" t="inlineStr">
+      <c r="F772" s="30" t="inlineStr">
         <is>
           <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
         </is>
@@ -44159,11 +44182,11 @@
       </c>
       <c r="C773" s="28" t="inlineStr">
         <is>
-          <t>cộng tác viên viết bài pr</t>
+          <t>tuyển ctv viết bài pr</t>
         </is>
       </c>
       <c r="D773" s="29" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E773" s="37" t="inlineStr">
         <is>
@@ -44185,7 +44208,7 @@
       </c>
       <c r="C774" s="28" t="inlineStr">
         <is>
-          <t>agency tuyển ctv viết bài pr</t>
+          <t>tuyển ctv viết bài pr báo chí</t>
         </is>
       </c>
       <c r="D774" s="29" t="n">
@@ -44211,7 +44234,7 @@
       </c>
       <c r="C775" s="28" t="inlineStr">
         <is>
-          <t>agency tuyển team viết bài pr</t>
+          <t>tuyển cộng tác viên viết bài pr</t>
         </is>
       </c>
       <c r="D775" s="29" t="n">
@@ -44237,7 +44260,7 @@
       </c>
       <c r="C776" s="28" t="inlineStr">
         <is>
-          <t>agency tuyển viết bài pr</t>
+          <t>tuyển người viết bài pr</t>
         </is>
       </c>
       <c r="D776" s="29" t="n">
@@ -44263,7 +44286,7 @@
       </c>
       <c r="C777" s="28" t="inlineStr">
         <is>
-          <t>mục đích đăng bài tuyển dụng để pr</t>
+          <t>tuyển nhân viên pr viết bài website</t>
         </is>
       </c>
       <c r="D777" s="29" t="n">
@@ -44289,7 +44312,7 @@
       </c>
       <c r="C778" s="28" t="inlineStr">
         <is>
-          <t>tuyển ctv viết bài pr</t>
+          <t>tuyển viết bài pr agency</t>
         </is>
       </c>
       <c r="D778" s="29" t="n">
@@ -44307,7 +44330,7 @@
       </c>
     </row>
     <row r="779">
-      <c r="A779" s="27" t="n"/>
+      <c r="A779" s="31" t="n"/>
       <c r="B779" s="28" t="inlineStr">
         <is>
           <t>—</t>
@@ -44315,7 +44338,7 @@
       </c>
       <c r="C779" s="28" t="inlineStr">
         <is>
-          <t>tuyển ctv viết bài pr báo chí</t>
+          <t>tuyển viết bài pr đăng báo</t>
         </is>
       </c>
       <c r="D779" s="29" t="n">
@@ -44333,160 +44356,160 @@
       </c>
     </row>
     <row r="780">
-      <c r="A780" s="27" t="n"/>
-      <c r="B780" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C780" s="28" t="inlineStr">
-        <is>
-          <t>tuyển cộng tác viên viết bài pr</t>
-        </is>
-      </c>
-      <c r="D780" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E780" s="37" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
-        </is>
-      </c>
-      <c r="F780" s="30" t="inlineStr">
-        <is>
-          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
+      <c r="A780" s="22" t="inlineStr">
+        <is>
+          <t>PR theo sự kiện</t>
+        </is>
+      </c>
+      <c r="B780" s="23" t="inlineStr">
+        <is>
+          <t>Từ khoá chính</t>
+        </is>
+      </c>
+      <c r="C780" s="23" t="inlineStr">
+        <is>
+          <t>viết bài pr cho sự kiện</t>
+        </is>
+      </c>
+      <c r="D780" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E780" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="F780" s="26" t="inlineStr">
+        <is>
+          <t>Mục con trong /bai-pr-mau/</t>
         </is>
       </c>
     </row>
     <row r="781">
       <c r="A781" s="27" t="n"/>
-      <c r="B781" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C781" s="28" t="inlineStr">
-        <is>
-          <t>tuyển người viết bài pr</t>
-        </is>
-      </c>
-      <c r="D781" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E781" s="37" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
-        </is>
-      </c>
-      <c r="F781" s="30" t="inlineStr">
-        <is>
-          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
+      <c r="B781" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C781" s="32" t="inlineStr">
+        <is>
+          <t>bài pr sau sự kiện</t>
+        </is>
+      </c>
+      <c r="D781" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E781" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="F781" s="34" t="inlineStr">
+        <is>
+          <t>Mục con trong /bai-pr-mau/</t>
         </is>
       </c>
     </row>
     <row r="782">
       <c r="A782" s="27" t="n"/>
-      <c r="B782" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C782" s="28" t="inlineStr">
-        <is>
-          <t>tuyển nhân viên pr viết bài website</t>
-        </is>
-      </c>
-      <c r="D782" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E782" s="37" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
-        </is>
-      </c>
-      <c r="F782" s="30" t="inlineStr">
-        <is>
-          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
+      <c r="B782" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C782" s="32" t="inlineStr">
+        <is>
+          <t>bài pr sự kiện</t>
+        </is>
+      </c>
+      <c r="D782" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E782" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="F782" s="34" t="inlineStr">
+        <is>
+          <t>Mục con trong /bai-pr-mau/</t>
         </is>
       </c>
     </row>
     <row r="783">
       <c r="A783" s="27" t="n"/>
-      <c r="B783" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C783" s="28" t="inlineStr">
-        <is>
-          <t>tuyển viết bài pr agency</t>
-        </is>
-      </c>
-      <c r="D783" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E783" s="37" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
-        </is>
-      </c>
-      <c r="F783" s="30" t="inlineStr">
-        <is>
-          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
+      <c r="B783" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C783" s="32" t="inlineStr">
+        <is>
+          <t>bài pr sự kiện về quốc tế thiếu nhi</t>
+        </is>
+      </c>
+      <c r="D783" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E783" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="F783" s="34" t="inlineStr">
+        <is>
+          <t>Mục con trong /bai-pr-mau/</t>
         </is>
       </c>
     </row>
     <row r="784">
-      <c r="A784" s="31" t="n"/>
-      <c r="B784" s="28" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C784" s="28" t="inlineStr">
-        <is>
-          <t>tuyển viết bài pr đăng báo</t>
-        </is>
-      </c>
-      <c r="D784" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E784" s="37" t="inlineStr">
-        <is>
-          <t>Ngoài phạm vi</t>
-        </is>
-      </c>
-      <c r="F784" s="30" t="inlineStr">
-        <is>
-          <t>Intent ứng tuyển, không phải khách mua dịch vụ</t>
+      <c r="A784" s="27" t="n"/>
+      <c r="B784" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C784" s="32" t="inlineStr">
+        <is>
+          <t>bài viết pr sự kiện</t>
+        </is>
+      </c>
+      <c r="D784" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E784" s="25" t="inlineStr">
+        <is>
+          <t>Đã phủ (cụm PR)</t>
+        </is>
+      </c>
+      <c r="F784" s="34" t="inlineStr">
+        <is>
+          <t>Mục con trong /bai-pr-mau/</t>
         </is>
       </c>
     </row>
     <row r="785">
-      <c r="A785" s="22" t="inlineStr">
-        <is>
-          <t>PR theo sự kiện</t>
-        </is>
-      </c>
-      <c r="B785" s="23" t="inlineStr">
-        <is>
-          <t>Từ khoá chính</t>
-        </is>
-      </c>
-      <c r="C785" s="23" t="inlineStr">
-        <is>
-          <t>viết bài pr cho sự kiện</t>
-        </is>
-      </c>
-      <c r="D785" s="24" t="n">
-        <v>10</v>
+      <c r="A785" s="27" t="n"/>
+      <c r="B785" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C785" s="32" t="inlineStr">
+        <is>
+          <t>bài viết pr sự kiện ô tô</t>
+        </is>
+      </c>
+      <c r="D785" s="33" t="n">
+        <v>0</v>
       </c>
       <c r="E785" s="25" t="inlineStr">
         <is>
           <t>Đã phủ (cụm PR)</t>
         </is>
       </c>
-      <c r="F785" s="26" t="inlineStr">
+      <c r="F785" s="34" t="inlineStr">
         <is>
           <t>Mục con trong /bai-pr-mau/</t>
         </is>
@@ -44501,7 +44524,7 @@
       </c>
       <c r="C786" s="32" t="inlineStr">
         <is>
-          <t>bài pr sau sự kiện</t>
+          <t>caác bài viết pr sự kiện</t>
         </is>
       </c>
       <c r="D786" s="33" t="n">
@@ -44527,7 +44550,7 @@
       </c>
       <c r="C787" s="32" t="inlineStr">
         <is>
-          <t>bài pr sự kiện</t>
+          <t>caách viết bài pr sự kiện</t>
         </is>
       </c>
       <c r="D787" s="33" t="n">
@@ -44553,7 +44576,7 @@
       </c>
       <c r="C788" s="32" t="inlineStr">
         <is>
-          <t>bài pr sự kiện về quốc tế thiếu nhi</t>
+          <t>các bài viết pr cho sự kiện</t>
         </is>
       </c>
       <c r="D788" s="33" t="n">
@@ -44571,7 +44594,7 @@
       </c>
     </row>
     <row r="789">
-      <c r="A789" s="27" t="n"/>
+      <c r="A789" s="31" t="n"/>
       <c r="B789" s="32" t="inlineStr">
         <is>
           <t>—</t>
@@ -44579,7 +44602,7 @@
       </c>
       <c r="C789" s="32" t="inlineStr">
         <is>
-          <t>bài viết pr sự kiện</t>
+          <t>những bài viết pr cho sự kiện ngày hội sách</t>
         </is>
       </c>
       <c r="D789" s="33" t="n">
@@ -44597,144 +44620,149 @@
       </c>
     </row>
     <row r="790">
-      <c r="A790" s="27" t="n"/>
-      <c r="B790" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C790" s="32" t="inlineStr">
-        <is>
-          <t>bài viết pr sự kiện ô tô</t>
-        </is>
-      </c>
-      <c r="D790" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E790" s="25" t="inlineStr">
-        <is>
-          <t>Đã phủ (cụm PR)</t>
-        </is>
-      </c>
-      <c r="F790" s="34" t="inlineStr">
-        <is>
-          <t>Mục con trong /bai-pr-mau/</t>
+      <c r="A790" s="22" t="inlineStr">
+        <is>
+          <t>PR cá nhân / doanh nhân qua báo chí</t>
+        </is>
+      </c>
+      <c r="B790" s="23" t="inlineStr">
+        <is>
+          <t>Từ khoá chính</t>
+        </is>
+      </c>
+      <c r="C790" s="23" t="inlineStr">
+        <is>
+          <t>bài pr bản thân</t>
+        </is>
+      </c>
+      <c r="D790" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E790" s="36" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="F790" s="26" t="inlineStr">
+        <is>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" s="27" t="n"/>
-      <c r="B791" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C791" s="32" t="inlineStr">
-        <is>
-          <t>caác bài viết pr sự kiện</t>
-        </is>
-      </c>
-      <c r="D791" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E791" s="25" t="inlineStr">
-        <is>
-          <t>Đã phủ (cụm PR)</t>
-        </is>
-      </c>
-      <c r="F791" s="34" t="inlineStr">
-        <is>
-          <t>Mục con trong /bai-pr-mau/</t>
+      <c r="B791" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C791" s="28" t="inlineStr">
+        <is>
+          <t>bài viết pr bản thân</t>
+        </is>
+      </c>
+      <c r="D791" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E791" s="36" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="F791" s="30" t="inlineStr">
+        <is>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
     <row r="792">
       <c r="A792" s="27" t="n"/>
-      <c r="B792" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C792" s="32" t="inlineStr">
-        <is>
-          <t>caách viết bài pr sự kiện</t>
-        </is>
-      </c>
-      <c r="D792" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E792" s="25" t="inlineStr">
-        <is>
-          <t>Đã phủ (cụm PR)</t>
-        </is>
-      </c>
-      <c r="F792" s="34" t="inlineStr">
-        <is>
-          <t>Mục con trong /bai-pr-mau/</t>
+      <c r="B792" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C792" s="28" t="inlineStr">
+        <is>
+          <t>bài viết pr về bản thân</t>
+        </is>
+      </c>
+      <c r="D792" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E792" s="36" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="F792" s="30" t="inlineStr">
+        <is>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
     <row r="793">
       <c r="A793" s="27" t="n"/>
-      <c r="B793" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C793" s="32" t="inlineStr">
-        <is>
-          <t>các bài viết pr cho sự kiện</t>
-        </is>
-      </c>
-      <c r="D793" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E793" s="25" t="inlineStr">
-        <is>
-          <t>Đã phủ (cụm PR)</t>
-        </is>
-      </c>
-      <c r="F793" s="34" t="inlineStr">
-        <is>
-          <t>Mục con trong /bai-pr-mau/</t>
+      <c r="B793" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C793" s="28" t="inlineStr">
+        <is>
+          <t>nhờ các facebook cá nhân viết bài pr</t>
+        </is>
+      </c>
+      <c r="D793" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E793" s="36" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="F793" s="30" t="inlineStr">
+        <is>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
     <row r="794">
       <c r="A794" s="31" t="n"/>
-      <c r="B794" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C794" s="32" t="inlineStr">
-        <is>
-          <t>những bài viết pr cho sự kiện ngày hội sách</t>
-        </is>
-      </c>
-      <c r="D794" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E794" s="25" t="inlineStr">
-        <is>
-          <t>Đã phủ (cụm PR)</t>
-        </is>
-      </c>
-      <c r="F794" s="34" t="inlineStr">
-        <is>
-          <t>Mục con trong /bai-pr-mau/</t>
+      <c r="B794" s="28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C794" s="28" t="inlineStr">
+        <is>
+          <t>yêu cầu về bài pr cá nhân</t>
+        </is>
+      </c>
+      <c r="D794" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E794" s="36" t="inlineStr">
+        <is>
+          <t>Gap - mở rộng bài cluster</t>
+        </is>
+      </c>
+      <c r="F794" s="30" t="inlineStr">
+        <is>
+          <t>Đọc lại là nhu cầu booking báo để PR cho chính cá nhân (doanh nhân/chuyên gia muốn lên báo) - KHÔNG phải viết CV xin việc. Nhắc như 1 đối tượng khách trong bài mới 'Dịch vụ Viết Bài PR' (mục A) hoặc mở rộng /bai-pr-mau/, CTA về /booking-bao-pr/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A764:A771"/>
-    <mergeCell ref="A785:A794"/>
+  <mergeCells count="15">
+    <mergeCell ref="A764:A766"/>
+    <mergeCell ref="A790:A794"/>
+    <mergeCell ref="A767:A779"/>
     <mergeCell ref="A565:A690"/>
     <mergeCell ref="A332:A398"/>
     <mergeCell ref="A2:A71"/>
     <mergeCell ref="A738:A756"/>
-    <mergeCell ref="A772:A784"/>
+    <mergeCell ref="A780:A789"/>
     <mergeCell ref="A757:A763"/>
     <mergeCell ref="A72:A331"/>
     <mergeCell ref="A551:A564"/>
@@ -44771,28 +44799,28 @@
     <row r="3">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>PR bản thân / xin việc (Jiko PR)</t>
+          <t>PR bản thân - xin việc/du học Nhật (Jiko PR)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="40" t="inlineStr">
         <is>
-          <t>8 tu khoa - 20 luot/thang</t>
+          <t>3 tu khoa - 20 luot/thang</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="41" t="inlineStr">
         <is>
-          <t>SERP là site tuyển dụng/du học, khác PR báo chí</t>
+          <t>Tự giới thiệu khi phỏng vấn/xin việc/du học Nhật (自己PR) hoặc game học tiếng Nhật - không liên quan báo chí/booking</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="42" t="inlineStr">
         <is>
-          <t>Vi du: bài mẫu pr bản thân bằng tiếng nhật, bài pr bản thân, bài pr bản thân bằng tiếng nhật, bài viết pr bản thân, bài viết pr về bản thân, các bài viết pr cho game học tiếng nhật, nhờ các facebook cá nhân viết bài pr, yêu cầu về bài pr cá nhân</t>
+          <t>Vi du: bài mẫu pr bản thân bằng tiếng nhật, bài pr bản thân bằng tiếng nhật, các bài viết pr cho game học tiếng nhật</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: session 2026-08-17 17:48
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/ke-hoach-noi-dung-cum-pr-2026-08-10.xlsx
+++ b/content/ke-hoach-noi-dung-cum-pr-2026-08-10.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +79,10 @@
     <font>
       <b val="1"/>
       <color rgb="006B7280"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -200,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -261,6 +265,20 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -627,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F791"/>
+  <dimension ref="A1:F845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10898,7 +10916,7 @@
       </c>
       <c r="B722" s="16" t="inlineStr">
         <is>
-          <t>PR doanh nghiệp / thương hiệu</t>
+          <t>PR thương hiệu lớn (mẫu bài)</t>
         </is>
       </c>
       <c r="C722" s="16" t="inlineStr">
@@ -10907,7 +10925,7 @@
         </is>
       </c>
       <c r="D722" s="17" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="E722" s="18" t="inlineStr">
         <is>
@@ -10919,10 +10937,24 @@
       </c>
     </row>
     <row r="723">
-      <c r="A723" s="20" t="n"/>
-      <c r="B723" s="20" t="n"/>
-      <c r="C723" s="20" t="n"/>
-      <c r="D723" s="20" t="n"/>
+      <c r="A723" s="23" t="inlineStr">
+        <is>
+          <t>CHƯA CÓ - cần viết mới</t>
+        </is>
+      </c>
+      <c r="B723" s="16" t="inlineStr">
+        <is>
+          <t>PR doanh nghiệp / công ty</t>
+        </is>
+      </c>
+      <c r="C723" s="16" t="inlineStr">
+        <is>
+          <t>CHƯA CÓ - viết bài mới "Cách viết bài PR cho doanh nghiệp/công ty" (howto): định nghĩa ngắn (link về /bai-pr-la-gi/, không lặp lại), các bước viết, ví dụ theo ngành (đại lý ô tô, may mặc, thiết kế nội thất, công ty con/tập đoàn), 1-2 ví dụ minh hoạ theo thương hiệu lớn (Honda, Nike - dán nhãn "ví dụ minh hoạ", không phải case thật), FAQ (giới hạn 200 từ, có được bán bài PR doanh nghiệp không). CTA về /booking-bao-pr/</t>
+        </is>
+      </c>
+      <c r="D723" s="17" t="n">
+        <v>70</v>
+      </c>
       <c r="E723" s="18" t="inlineStr">
         <is>
           <t>bài pr doanh nghiệp</t>
@@ -11271,7 +11303,7 @@
     <row r="747">
       <c r="A747" s="20" t="n"/>
       <c r="B747" s="20" t="n"/>
-      <c r="C747" s="20" t="n"/>
+      <c r="C747" s="21" t="n"/>
       <c r="D747" s="20" t="n"/>
       <c r="E747" s="18" t="inlineStr">
         <is>
@@ -11285,7 +11317,11 @@
     <row r="748">
       <c r="A748" s="20" t="n"/>
       <c r="B748" s="20" t="n"/>
-      <c r="C748" s="20" t="n"/>
+      <c r="C748" s="16" t="inlineStr">
+        <is>
+          <t>Đã có bài (bài con riêng) - /lead-bai-pr-la-gi/ (mở rộng chi tiết từ /bai-pr-la-gi/, viết 2026-08-11)</t>
+        </is>
+      </c>
       <c r="D748" s="20" t="n"/>
       <c r="E748" s="18" t="inlineStr">
         <is>
@@ -11299,7 +11335,7 @@
     <row r="749">
       <c r="A749" s="20" t="n"/>
       <c r="B749" s="20" t="n"/>
-      <c r="C749" s="20" t="n"/>
+      <c r="C749" s="16" t="n"/>
       <c r="D749" s="20" t="n"/>
       <c r="E749" s="18" t="inlineStr">
         <is>
@@ -11397,7 +11433,7 @@
     <row r="756">
       <c r="A756" s="20" t="n"/>
       <c r="B756" s="20" t="n"/>
-      <c r="C756" s="20" t="n"/>
+      <c r="C756" s="21" t="n"/>
       <c r="D756" s="20" t="n"/>
       <c r="E756" s="18" t="inlineStr">
         <is>
@@ -11411,7 +11447,11 @@
     <row r="757">
       <c r="A757" s="20" t="n"/>
       <c r="B757" s="20" t="n"/>
-      <c r="C757" s="20" t="n"/>
+      <c r="C757" s="16" t="inlineStr">
+        <is>
+          <t>Đã có bài (bài con riêng) - /sapo-la-gi-trong-bai-pr/ (vị trí/vai trò/format sapo, viết 2026-08-11)</t>
+        </is>
+      </c>
       <c r="D757" s="20" t="n"/>
       <c r="E757" s="18" t="inlineStr">
         <is>
@@ -11425,7 +11465,7 @@
     <row r="758">
       <c r="A758" s="20" t="n"/>
       <c r="B758" s="20" t="n"/>
-      <c r="C758" s="20" t="n"/>
+      <c r="C758" s="16" t="n"/>
       <c r="D758" s="20" t="n"/>
       <c r="E758" s="18" t="inlineStr">
         <is>
@@ -11940,52 +11980,651 @@
         <v>0</v>
       </c>
     </row>
+    <row r="792">
+      <c r="A792" s="25" t="inlineStr">
+        <is>
+          <t>Có bài, cần bổ sung thêm</t>
+        </is>
+      </c>
+      <c r="B792" s="26" t="inlineStr">
+        <is>
+          <t>Công thức viết bài PR: PAS / 3S / Strings</t>
+        </is>
+      </c>
+      <c r="C792" s="26" t="inlineStr">
+        <is>
+          <t>Bổ sung 3 mục lớn (PAS, 3S, Strings) vào /cach-viet-bai-pr-chuan-bao-chi/ - moi cong thuc 1 so do giai thich + vi du bai PR mau ap dung. 'công thức pas' rieng le da 260 vol (cao hon volume ca cum hien tai 280) - CAN research SERP truoc khi quyet dinh giu lam muc con hay tach trang rieng /cong-thuc-pas-la-gi/ (theo audit-intent-truoc.md, khong tu quyet)</t>
+        </is>
+      </c>
+      <c r="D792" s="27" t="n">
+        <v>430</v>
+      </c>
+      <c r="E792" s="28" t="inlineStr">
+        <is>
+          <t>công thức pas</t>
+        </is>
+      </c>
+      <c r="F792" s="28" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="E793" s="28" t="inlineStr">
+        <is>
+          <t>công thức content pas</t>
+        </is>
+      </c>
+      <c r="F793" s="28" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="E794" s="28" t="inlineStr">
+        <is>
+          <t>công thức pas là gì</t>
+        </is>
+      </c>
+      <c r="F794" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="E795" s="28" t="inlineStr">
+        <is>
+          <t>công thức viết bài pas</t>
+        </is>
+      </c>
+      <c r="F795" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="E796" s="28" t="inlineStr">
+        <is>
+          <t>công thức viết content pas</t>
+        </is>
+      </c>
+      <c r="F796" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="E797" s="28" t="inlineStr">
+        <is>
+          <t>cách viết công thức pas</t>
+        </is>
+      </c>
+      <c r="F797" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="E798" s="28" t="inlineStr">
+        <is>
+          <t>công thức bán hàng pas</t>
+        </is>
+      </c>
+      <c r="F798" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="E799" s="28" t="inlineStr">
+        <is>
+          <t>công thức 3s</t>
+        </is>
+      </c>
+      <c r="F799" s="28" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="E800" s="28" t="inlineStr">
+        <is>
+          <t>công thức strings</t>
+        </is>
+      </c>
+      <c r="F800" s="28" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="E801" s="28" t="inlineStr">
+        <is>
+          <t>ví dụ công thức strings</t>
+        </is>
+      </c>
+      <c r="F801" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="E802" s="28" t="inlineStr">
+        <is>
+          <t>ví dụ công thức strings pr</t>
+        </is>
+      </c>
+      <c r="F802" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="E803" s="28" t="inlineStr">
+        <is>
+          <t>công thức strings các bài viết theo công thức này</t>
+        </is>
+      </c>
+      <c r="F803" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="29" t="inlineStr">
+        <is>
+          <t>CHƯA CÓ - cần viết mới</t>
+        </is>
+      </c>
+      <c r="B804" s="26" t="inlineStr">
+        <is>
+          <t>Các dạng bài PR: Advertorial / Editorial / Testimonial</t>
+        </is>
+      </c>
+      <c r="C804" s="26" t="inlineStr">
+        <is>
+          <t>CHUA CO - viet bai moi 'Cac Dang Bai PR Pho Bien' giai thich + vi du mau tung dang (Advertorial/Editorial/Testimonial). Link 2 chieu voi /cach-viet-bai-pr-chuan-bao-chi/ (muc 'cac dang bai pr' dang chung chung, doi sang tro bai nay) va /bai-pr-mau/. CTA ve /booking-bao-pr/</t>
+        </is>
+      </c>
+      <c r="D804" s="27" t="n">
+        <v>160</v>
+      </c>
+      <c r="E804" s="28" t="inlineStr">
+        <is>
+          <t>bài advertorial</t>
+        </is>
+      </c>
+      <c r="F804" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="E805" s="28" t="inlineStr">
+        <is>
+          <t>bài advertorial mẫu</t>
+        </is>
+      </c>
+      <c r="F805" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="E806" s="28" t="inlineStr">
+        <is>
+          <t>bài advertorial mẫu về khách sạn</t>
+        </is>
+      </c>
+      <c r="F806" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="E807" s="28" t="inlineStr">
+        <is>
+          <t>cách viết bài advertorial</t>
+        </is>
+      </c>
+      <c r="F807" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="E808" s="28" t="inlineStr">
+        <is>
+          <t>viết bài advertorial</t>
+        </is>
+      </c>
+      <c r="F808" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="E809" s="28" t="inlineStr">
+        <is>
+          <t>viết bài advertorial cho bitis hunter x</t>
+        </is>
+      </c>
+      <c r="F809" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="E810" s="28" t="inlineStr">
+        <is>
+          <t>đăng bài advertorial</t>
+        </is>
+      </c>
+      <c r="F810" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="E811" s="28" t="inlineStr">
+        <is>
+          <t>bài editorial mẫu</t>
+        </is>
+      </c>
+      <c r="F811" s="28" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="E812" s="28" t="inlineStr">
+        <is>
+          <t>bài viết editorial</t>
+        </is>
+      </c>
+      <c r="F812" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="E813" s="28" t="inlineStr">
+        <is>
+          <t>dạng bài editorial</t>
+        </is>
+      </c>
+      <c r="F813" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="E814" s="28" t="inlineStr">
+        <is>
+          <t>bài editorial</t>
+        </is>
+      </c>
+      <c r="F814" s="28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="E815" s="28" t="inlineStr">
+        <is>
+          <t>bài báo editorial</t>
+        </is>
+      </c>
+      <c r="F815" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="E816" s="28" t="inlineStr">
+        <is>
+          <t>bài báo viết theo dạng editorial</t>
+        </is>
+      </c>
+      <c r="F816" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="E817" s="28" t="inlineStr">
+        <is>
+          <t>bài editorial kinh tế</t>
+        </is>
+      </c>
+      <c r="F817" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="E818" s="28" t="inlineStr">
+        <is>
+          <t>bài editorials</t>
+        </is>
+      </c>
+      <c r="F818" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="E819" s="28" t="inlineStr">
+        <is>
+          <t>các bài báo editorial</t>
+        </is>
+      </c>
+      <c r="F819" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="E820" s="28" t="inlineStr">
+        <is>
+          <t>các bài editorial về dịch vụ du lịch</t>
+        </is>
+      </c>
+      <c r="F820" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="E821" s="28" t="inlineStr">
+        <is>
+          <t>các bài viết editorial</t>
+        </is>
+      </c>
+      <c r="F821" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="E822" s="28" t="inlineStr">
+        <is>
+          <t>các dạng bài editorial</t>
+        </is>
+      </c>
+      <c r="F822" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="E823" s="28" t="inlineStr">
+        <is>
+          <t>những bài editorial hay nhất</t>
+        </is>
+      </c>
+      <c r="F823" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="E824" s="28" t="inlineStr">
+        <is>
+          <t>viết bài editorial</t>
+        </is>
+      </c>
+      <c r="F824" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="E825" s="28" t="inlineStr">
+        <is>
+          <t>viết bài editorial và advertorial</t>
+        </is>
+      </c>
+      <c r="F825" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="E826" s="28" t="inlineStr">
+        <is>
+          <t>ví dụ bài editorial</t>
+        </is>
+      </c>
+      <c r="F826" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="E827" s="28" t="inlineStr">
+        <is>
+          <t>dạng bài testimonial</t>
+        </is>
+      </c>
+      <c r="F827" s="28" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="E828" s="28" t="inlineStr">
+        <is>
+          <t>bài viết testimonial hay</t>
+        </is>
+      </c>
+      <c r="F828" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="E829" s="28" t="inlineStr">
+        <is>
+          <t>dạng bài testimonial là gì</t>
+        </is>
+      </c>
+      <c r="F829" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="25" t="inlineStr">
+        <is>
+          <t>Có bài, cần bổ sung thêm</t>
+        </is>
+      </c>
+      <c r="B830" s="26" t="inlineStr">
+        <is>
+          <t>Mô hình kim tự tháp ngược trong viết bài PR</t>
+        </is>
+      </c>
+      <c r="C830" s="26" t="inlineStr">
+        <is>
+          <t>Them 1 muc ngan + so do minh hoa 'Mo hinh kim tu thap nguoc' vao /cach-viet-bai-pr-chuan-bao-chi/ (muc cau truc bai, da co dong 0-vol 'mo hinh kim tu thap nguoc trong viet bai pr'). CANH BAO: 'mo hinh kim tu thap nguoc' (50) va 'kim tu thap nguoc' (10) la tu khoa DA NGHIA - phan lon volume thuoc ve bao tang/landmark Ha Noi va mo hinh tai chinh John Exter (xem cum ben duoi), KHONG phai khai niem viet bai. KHONG viet bai/pillar rieng cho cum nay, chi la 1 muc bo sung, khong ky vong volume thuc te cao nhu con so hien</t>
+        </is>
+      </c>
+      <c r="D830" s="27" t="n">
+        <v>60</v>
+      </c>
+      <c r="E830" s="28" t="inlineStr">
+        <is>
+          <t>mô hình kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F830" s="28" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="E831" s="28" t="inlineStr">
+        <is>
+          <t>kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F831" s="28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="E832" s="28" t="inlineStr">
+        <is>
+          <t>kim tự tháp ngược trong viết content</t>
+        </is>
+      </c>
+      <c r="F832" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="E833" s="28" t="inlineStr">
+        <is>
+          <t>format chuẩn kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F833" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="E834" s="28" t="inlineStr">
+        <is>
+          <t>đây là mô hình kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F834" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="30" t="inlineStr">
+        <is>
+          <t>Không viết (ngoài phạm vi)</t>
+        </is>
+      </c>
+      <c r="B835" s="26" t="inlineStr">
+        <is>
+          <t>Kim tự tháp ngược - bảo tàng / mô hình tài chính</t>
+        </is>
+      </c>
+      <c r="C835" s="26" t="inlineStr">
+        <is>
+          <t>Ngoai pham vi - thuoc chu de bao tang/landmark kien truc (Ha Noi) hoac mo hinh tai chinh John Exter (lai suat, thanh khoan ngan hang), khong lien quan viet bai PR/content</t>
+        </is>
+      </c>
+      <c r="D835" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E835" s="28" t="inlineStr">
+        <is>
+          <t>bảo tàng kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F835" s="28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="E836" s="28" t="inlineStr">
+        <is>
+          <t>bảo tàng hình kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F836" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="E837" s="28" t="inlineStr">
+        <is>
+          <t>bảo tàng kim tự tháp lộn ngược</t>
+        </is>
+      </c>
+      <c r="F837" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="E838" s="28" t="inlineStr">
+        <is>
+          <t>kim tự tháp chổng ngược ở hà nội</t>
+        </is>
+      </c>
+      <c r="F838" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="E839" s="28" t="inlineStr">
+        <is>
+          <t>kim tự tháp ngược ở hà nội</t>
+        </is>
+      </c>
+      <c r="F839" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="E840" s="28" t="inlineStr">
+        <is>
+          <t>lãi suất mô hình kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F840" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="E841" s="28" t="inlineStr">
+        <is>
+          <t>lãi suất ngân hàng mô hình kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F841" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="E842" s="28" t="inlineStr">
+        <is>
+          <t>mô hình kim tự tháp ngược của john exter</t>
+        </is>
+      </c>
+      <c r="F842" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="E843" s="28" t="inlineStr">
+        <is>
+          <t>mô hình kim tự tháp ngược john exter</t>
+        </is>
+      </c>
+      <c r="F843" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="E844" s="28" t="inlineStr">
+        <is>
+          <t>mô hình kim tự tháp ngược lãi suất</t>
+        </is>
+      </c>
+      <c r="F844" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="E845" s="28" t="inlineStr">
+        <is>
+          <t>mô hình quản trị kim tự tháp ngược</t>
+        </is>
+      </c>
+      <c r="F845" s="28" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="62">
     <mergeCell ref="D566:D647"/>
+    <mergeCell ref="D23:D41"/>
+    <mergeCell ref="B298:B366"/>
     <mergeCell ref="D167:D297"/>
+    <mergeCell ref="C749:C756"/>
+    <mergeCell ref="D298:D366"/>
     <mergeCell ref="D771:D773"/>
+    <mergeCell ref="B42:B48"/>
     <mergeCell ref="D761:D770"/>
+    <mergeCell ref="D648:D721"/>
+    <mergeCell ref="C746:C747"/>
+    <mergeCell ref="B723:B745"/>
+    <mergeCell ref="A761:A770"/>
     <mergeCell ref="A648:A721"/>
+    <mergeCell ref="C761:C770"/>
     <mergeCell ref="C367:C565"/>
+    <mergeCell ref="B49:B53"/>
+    <mergeCell ref="A746:A760"/>
+    <mergeCell ref="A167:A297"/>
+    <mergeCell ref="C298:C366"/>
+    <mergeCell ref="A42:A48"/>
+    <mergeCell ref="A771:A773"/>
+    <mergeCell ref="C723:C745"/>
+    <mergeCell ref="C758:C760"/>
+    <mergeCell ref="C648:C721"/>
     <mergeCell ref="B771:B773"/>
     <mergeCell ref="A774:A791"/>
     <mergeCell ref="B54:B166"/>
     <mergeCell ref="D42:D48"/>
+    <mergeCell ref="C774:C791"/>
     <mergeCell ref="D54:D166"/>
-    <mergeCell ref="C774:C791"/>
-    <mergeCell ref="A54:A166"/>
-    <mergeCell ref="C42:C48"/>
-    <mergeCell ref="C54:C166"/>
-    <mergeCell ref="B746:B760"/>
-    <mergeCell ref="D746:D760"/>
-    <mergeCell ref="D774:D791"/>
-    <mergeCell ref="A298:A366"/>
-    <mergeCell ref="A566:A647"/>
-    <mergeCell ref="C566:C647"/>
-    <mergeCell ref="B722:B745"/>
-    <mergeCell ref="B774:B791"/>
-    <mergeCell ref="D722:D745"/>
-    <mergeCell ref="C2:C22"/>
-    <mergeCell ref="B648:B721"/>
-    <mergeCell ref="B761:B770"/>
-    <mergeCell ref="A722:A745"/>
-    <mergeCell ref="D23:D41"/>
-    <mergeCell ref="B298:B366"/>
-    <mergeCell ref="D298:D366"/>
-    <mergeCell ref="B42:B48"/>
-    <mergeCell ref="D648:D721"/>
-    <mergeCell ref="A761:A770"/>
-    <mergeCell ref="C761:C770"/>
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="A746:A760"/>
-    <mergeCell ref="A167:A297"/>
-    <mergeCell ref="C746:C760"/>
-    <mergeCell ref="C298:C366"/>
-    <mergeCell ref="A42:A48"/>
-    <mergeCell ref="A771:A773"/>
-    <mergeCell ref="C648:C721"/>
-    <mergeCell ref="C722:C745"/>
     <mergeCell ref="B2:B22"/>
     <mergeCell ref="A49:A53"/>
     <mergeCell ref="D2:D22"/>
@@ -11993,11 +12632,26 @@
     <mergeCell ref="B566:B647"/>
     <mergeCell ref="B167:B297"/>
     <mergeCell ref="A367:A565"/>
+    <mergeCell ref="A54:A166"/>
     <mergeCell ref="B23:B41"/>
+    <mergeCell ref="C42:C48"/>
+    <mergeCell ref="C54:C166"/>
+    <mergeCell ref="B746:B760"/>
+    <mergeCell ref="D746:D760"/>
+    <mergeCell ref="D774:D791"/>
+    <mergeCell ref="A723:A745"/>
     <mergeCell ref="A2:A22"/>
     <mergeCell ref="D49:D53"/>
+    <mergeCell ref="D723:D745"/>
     <mergeCell ref="C167:C297"/>
     <mergeCell ref="C771:C773"/>
+    <mergeCell ref="A298:A366"/>
+    <mergeCell ref="A566:A647"/>
+    <mergeCell ref="C566:C647"/>
+    <mergeCell ref="B774:B791"/>
+    <mergeCell ref="C2:C22"/>
+    <mergeCell ref="B648:B721"/>
+    <mergeCell ref="B761:B770"/>
     <mergeCell ref="B367:B565"/>
     <mergeCell ref="A23:A41"/>
     <mergeCell ref="D367:D565"/>

</xml_diff>